<commit_message>
feat: added position and draft plan. need to account for injuries
</commit_message>
<xml_diff>
--- a/output/top100_by_position.xlsx
+++ b/output/top100_by_position.xlsx
@@ -18772,12 +18772,12 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Deuce Vaughn</t>
+          <t>Jeff Wilson</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>DAL</t>
+          <t>SF</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
@@ -18786,7 +18786,7 @@
         </is>
       </c>
       <c r="D100" t="n">
-        <v>21.853</v>
+        <v>23.049</v>
       </c>
       <c r="E100" t="n">
         <v>0</v>
@@ -18798,19 +18798,19 @@
         <v>0</v>
       </c>
       <c r="H100" t="n">
-        <v>44.23</v>
+        <v>57.09</v>
       </c>
       <c r="I100" t="n">
-        <v>0.33</v>
+        <v>0.48</v>
       </c>
       <c r="J100" t="n">
-        <v>2.93</v>
+        <v>2.36</v>
       </c>
       <c r="K100" t="n">
-        <v>22.6</v>
+        <v>17.1</v>
       </c>
       <c r="L100" t="n">
-        <v>0.06</v>
+        <v>0.09</v>
       </c>
       <c r="M100" t="n">
         <v>0</v>
@@ -18822,7 +18822,7 @@
         <v>0</v>
       </c>
       <c r="P100" t="n">
-        <v>0.02</v>
+        <v>0.03</v>
       </c>
       <c r="Q100" t="n">
         <v>0</v>
@@ -18879,18 +18879,18 @@
         <v>0</v>
       </c>
       <c r="AI100" t="n">
-        <v>37</v>
+        <v>88</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Sione Vaki</t>
+          <t>Deuce Vaughn</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>DET</t>
+          <t>DAL</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
@@ -18899,7 +18899,7 @@
         </is>
       </c>
       <c r="D101" t="n">
-        <v>20.582</v>
+        <v>21.853</v>
       </c>
       <c r="E101" t="n">
         <v>0</v>
@@ -18911,32 +18911,32 @@
         <v>0</v>
       </c>
       <c r="H101" t="n">
-        <v>47.86</v>
+        <v>44.23</v>
       </c>
       <c r="I101" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="J101" t="n">
+        <v>2.93</v>
+      </c>
+      <c r="K101" t="n">
+        <v>22.6</v>
+      </c>
+      <c r="L101" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="M101" t="n">
+        <v>0</v>
+      </c>
+      <c r="N101" t="n">
+        <v>0</v>
+      </c>
+      <c r="O101" t="n">
+        <v>0</v>
+      </c>
+      <c r="P101" t="n">
         <v>0.02</v>
       </c>
-      <c r="J101" t="n">
-        <v>3.18</v>
-      </c>
-      <c r="K101" t="n">
-        <v>24.46</v>
-      </c>
-      <c r="L101" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="M101" t="n">
-        <v>0</v>
-      </c>
-      <c r="N101" t="n">
-        <v>0</v>
-      </c>
-      <c r="O101" t="n">
-        <v>0</v>
-      </c>
-      <c r="P101" t="n">
-        <v>0</v>
-      </c>
       <c r="Q101" t="n">
         <v>0</v>
       </c>
@@ -18992,7 +18992,7 @@
         <v>0</v>
       </c>
       <c r="AI101" t="n">
-        <v>129</v>
+        <v>37</v>
       </c>
     </row>
   </sheetData>
@@ -38482,7 +38482,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>PHI</t>
+          <t>HOU</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -49317,7 +49317,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="C3" t="n">
         <v>0</v>
@@ -49329,19 +49329,19 @@
         <v>0</v>
       </c>
       <c r="F3" t="n">
+        <v>120</v>
+      </c>
+      <c r="G3" t="n">
         <v>116</v>
       </c>
-      <c r="G3" t="n">
-        <v>112</v>
-      </c>
       <c r="H3" t="n">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="I3" t="n">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="J3" t="n">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="K3" t="n">
         <v>5</v>
@@ -49353,7 +49353,7 @@
         <v>0</v>
       </c>
       <c r="N3" t="n">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="O3" t="n">
         <v>0</v>
@@ -49410,7 +49410,7 @@
         <v>0</v>
       </c>
       <c r="AG3" t="n">
-        <v>117</v>
+        <v>121</v>
       </c>
     </row>
     <row r="4">
@@ -49420,7 +49420,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="C4" t="n">
         <v>1</v>
@@ -49438,13 +49438,13 @@
         <v>47</v>
       </c>
       <c r="H4" t="n">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="I4" t="n">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="J4" t="n">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="K4" t="n">
         <v>44</v>
@@ -49513,7 +49513,7 @@
         <v>0</v>
       </c>
       <c r="AG4" t="n">
-        <v>183</v>
+        <v>184</v>
       </c>
     </row>
     <row r="5">

</xml_diff>